<commit_message>
updated init file CalSim3DataExtractionInitFile_v4.xlsx
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADB0EF7-E2DC-4AA8-8571-73D6C2E802E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAE7406-5552-4B8B-B291-2B775D0CEF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12510" yWindow="-18345" windowWidth="17460" windowHeight="15525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8385" yWindow="-16050" windowWidth="29070" windowHeight="16470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
@@ -238,7 +238,7 @@
     <t>E220</t>
   </si>
   <si>
-    <t>E240</t>
+    <t>E242</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
modified init file to extend to new scenario 19
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
+++ b/notebooks/CalSim3DataExtractionInitFile_v4.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAE7406-5552-4B8B-B291-2B775D0CEF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D42193-6ED7-4972-959B-347C5CB4422B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8385" yWindow="-16050" windowWidth="29070" windowHeight="16470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Init" sheetId="1" r:id="rId1"/>
@@ -190,27 +190,6 @@
     <t>trend_report_variables_v5.xlsx</t>
   </si>
   <si>
-    <t>A18</t>
-  </si>
-  <si>
-    <t>B18</t>
-  </si>
-  <si>
-    <t>C18</t>
-  </si>
-  <si>
-    <t>G18</t>
-  </si>
-  <si>
-    <t>H18</t>
-  </si>
-  <si>
-    <t>I18</t>
-  </si>
-  <si>
-    <t>J18</t>
-  </si>
-  <si>
     <t>Inflows Extraction Dir</t>
   </si>
   <si>
@@ -239,6 +218,27 @@
   </si>
   <si>
     <t>E242</t>
+  </si>
+  <si>
+    <t>A19</t>
+  </si>
+  <si>
+    <t>B19</t>
+  </si>
+  <si>
+    <t>C19</t>
+  </si>
+  <si>
+    <t>G19</t>
+  </si>
+  <si>
+    <t>H19</t>
+  </si>
+  <si>
+    <t>I19</t>
+  </si>
+  <si>
+    <t>J19</t>
   </si>
 </sst>
 </file>
@@ -632,7 +632,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -646,7 +646,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -660,7 +660,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -674,7 +674,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -688,7 +688,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -702,7 +702,7 @@
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -716,7 +716,7 @@
         <v>37</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -754,7 +754,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -821,26 +821,26 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -848,13 +848,13 @@
         <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>